<commit_message>
chore(refs): update NotesTabContents_BuyerFirst.xlsx baseline
Track the current sheet so future edits surface as diffs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proxybuying-obsidian/AI-Context/references/NotesTabContents_BuyerFirst.xlsx
+++ b/proxybuying-obsidian/AI-Context/references/NotesTabContents_BuyerFirst.xlsx
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="274">
   <si>
     <t xml:space="preserve">NOTES TABS AND EMAILS CONTENT</t>
   </si>
@@ -237,7 +237,7 @@
   </si>
   <si>
     <t xml:space="preserve">✉ Estimate accepted for order {ref}
-The buyer has accepted your estimate for order {ref} ({route}). The order is now open on the Queuing Cargo board for a Carrier to offer. [Button: View the order]</t>
+The buyer has accepted your estimate for order {ref} ({route}). The order is now listed on "Buyer's Cargo List" for a Traveler to offer. [Button: View the order]</t>
   </si>
   <si>
     <t>[3A.0B]</t>
@@ -493,7 +493,7 @@
     <t xml:space="preserve">* Make sure to select the correct Shipment Option (Pick Up or Request Reship). If you select Reship, you will pay for Reshipment cost directly to the traveler</t>
   </si>
   <si>
-    <t xml:space="preserve">* After you click “Send Cargo Order”, the Order will be listed on "3. Queuing Buyer's Cargo" .</t>
+    <t xml:space="preserve">* After you click “Send Cargo Order”, the Order will be listed on "Buyer's Cargo List" .</t>
   </si>
   <si>
     <t xml:space="preserve">* You still can edit this Order later before a traveler send an Offer and you accept it.</t>
@@ -502,13 +502,16 @@
     <t xml:space="preserve">* Traveler who will carry this package has the right to open the box/luggage to verify the content.</t>
   </si>
   <si>
+    <t xml:space="preserve">[1A.1BC] -&gt; [B1.1BC]</t>
+  </si>
+  <si>
     <t>[1A.1BC]</t>
   </si>
   <si>
     <t xml:space="preserve">Send Cargo Order</t>
   </si>
   <si>
-    <t xml:space="preserve">Your cargo order has been listed on "3. Queuing Buyer's Cargo" awaiting for traveler to send an offer.</t>
+    <t xml:space="preserve">Your cargo order has been listed on "Buyer's Cargo List" awaiting for traveler to send an offer.</t>
   </si>
   <si>
     <t xml:space="preserve">✉ We received your order {ref}
@@ -528,7 +531,7 @@
     <t>Edit</t>
   </si>
   <si>
-    <t xml:space="preserve">Your cargo order has been listed on "3. Queuing Buyer's Cargo", please Save Changes after making any updates.</t>
+    <t xml:space="preserve">Your cargo order has been listed on "Buyer's Cargo List", please Save Changes after making any updates.</t>
   </si>
   <si>
     <t>[1A.3BC]</t>
@@ -925,7 +928,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd-mmm"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -954,6 +957,12 @@
     <font>
       <sz val="11.000000"/>
       <color indexed="2"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.000000"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -1002,7 +1011,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="13">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -1059,7 +1068,7 @@
       <top style="thin">
         <color theme="1"/>
       </top>
-      <bottom/>
+      <bottom style="none"/>
       <diagonal style="none"/>
     </border>
     <border>
@@ -1073,19 +1082,6 @@
       <bottom style="thin">
         <color theme="1"/>
       </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom style="none"/>
       <diagonal style="none"/>
     </border>
     <border>
@@ -1124,31 +1120,7 @@
       <right style="thin">
         <color theme="1"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
       <top style="none"/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color theme="1"/>
       </bottom>
@@ -1177,17 +1149,6 @@
       <diagonal style="none"/>
     </border>
     <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="none"/>
       <right style="none"/>
       <top style="none"/>
@@ -1200,7 +1161,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="96">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center"/>
@@ -1210,12 +1171,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
@@ -1252,45 +1207,42 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="1" pivotButton="0"/>
+    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
     <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
+    <xf fontId="0" fillId="0" borderId="8" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
+    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="1" pivotButton="0"/>
-    <xf fontId="0" fillId="0" borderId="8" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
-    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+    <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
-    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="1" pivotButton="0"/>
-    <xf fontId="0" fillId="0" borderId="11" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="11" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment vertical="center"/>
+    <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="1" pivotButton="0"/>
+    <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
+    <xf fontId="0" fillId="4" borderId="9" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="11" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
-    <xf fontId="0" fillId="0" borderId="12" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="1" pivotButton="0"/>
-    <xf fontId="0" fillId="0" borderId="13" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
-    <xf fontId="0" fillId="4" borderId="11" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="14" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
     <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
@@ -1301,16 +1253,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="5" borderId="11" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+    <xf fontId="0" fillId="5" borderId="9" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1321,118 +1267,99 @@
     <xf fontId="0" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
     <xf fontId="0" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="11" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+    <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="9" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="6" borderId="4" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="6" borderId="4" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="7" borderId="4" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="6" borderId="4" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="12" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
+    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="4" borderId="9" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="5" borderId="9" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+    <xf fontId="0" fillId="7" borderId="9" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="5" borderId="11" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="6" borderId="6" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="6" borderId="6" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="7" borderId="4" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="6" borderId="6" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="15" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="7" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="15" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
-    <xf fontId="0" fillId="0" borderId="16" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
-    <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
-    <xf fontId="0" fillId="0" borderId="12" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="0" pivotButton="0"/>
-    <xf fontId="0" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="7" borderId="11" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="6" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+    <xf fontId="3" fillId="6" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
@@ -1441,24 +1368,21 @@
     <xf fontId="1" fillId="7" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="4" fillId="6" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+    <xf fontId="4" fillId="6" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" quotePrefix="1" pivotButton="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="1" pivotButton="0">
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="1" pivotButton="0"/>
+    <xf fontId="5" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" quotePrefix="1" pivotButton="0"/>
-    <xf fontId="3" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+    <xf fontId="5" fillId="7" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="3" fillId="7" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="4" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" quotePrefix="0" pivotButton="0"/>
-    <xf fontId="4" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" quotePrefix="0" pivotButton="0"/>
+    <xf fontId="2" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" quotePrefix="0" pivotButton="0"/>
+    <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" quotePrefix="0" pivotButton="0"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center"/>
     </xf>
@@ -1468,9 +1392,6 @@
     <xf fontId="0" fillId="0" borderId="4" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" quotePrefix="1" pivotButton="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" quotePrefix="1" pivotButton="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1489,7 +1410,6 @@
     <xf fontId="3" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1506,8 +1426,8 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="tc={CFFA49ED-4450-354E-22CF-5ACF75A6C676}" id="{5AEB340D-F449-F7F0-3302-707B577426DC}"/>
-  <person displayName="tc={1959D02E-70EF-64B2-D914-FFD88B3CE95E}" id="{441A3A53-725A-F159-8612-D3F939113813}"/>
+  <person displayName="tc={CFFA49ED-4450-354E-22CF-5ACF75A6C676}" id="{5E3E41C2-777B-D7EA-DFDC-C96F34604B6D}"/>
+  <person displayName="tc={1959D02E-70EF-64B2-D914-FFD88B3CE95E}" id="{89FD70E1-AEAC-1068-5CD5-882CBF02EEE6}"/>
 </personList>
 </file>
 
@@ -1991,12 +1911,12 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="F21" personId="{5AEB340D-F449-F7F0-3302-707B577426DC}" id="{68CDCEE9-3798-4095-B2EA-7F25D17F7713}" done="0">
+  <threadedComment ref="F21" personId="{5E3E41C2-777B-D7EA-DFDC-C96F34604B6D}" id="{68CDCEE9-3798-4095-B2EA-7F25D17F7713}" done="0">
     <text xml:space="preserve">opa:
 Update wordings
 </text>
   </threadedComment>
-  <threadedComment ref="J21" personId="{441A3A53-725A-F159-8612-D3F939113813}" id="{31134796-9E39-40A0-9686-BD15732127D7}" done="0">
+  <threadedComment ref="J21" personId="{89FD70E1-AEAC-1068-5CD5-882CBF02EEE6}" id="{31134796-9E39-40A0-9686-BD15732127D7}" done="0">
     <text xml:space="preserve">opa:
 Update wordings
 </text>
@@ -2012,10 +1932,12 @@
   </sheetPr>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="2" style="1" width="7.7109375"/>
+    <col customWidth="1" min="1" max="1" style="1" width="5.421875"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" style="1" width="5.421875"/>
+    <col bestFit="1" min="3" max="3" width="5.421875"/>
     <col customWidth="1" min="4" max="4" style="2" width="9.00390625"/>
-    <col customWidth="1" min="5" max="5" style="3" width="20.7109375"/>
-    <col customWidth="1" min="6" max="8" style="2" width="25.7109375"/>
+    <col customWidth="1" min="5" max="5" style="3" width="19.00390625"/>
+    <col customWidth="1" min="6" max="8" style="2" width="26.7109375"/>
     <col customWidth="1" min="10" max="12" style="2" width="40.7109375"/>
     <col customWidth="1" min="13" max="14" style="2" width="30.57421875"/>
   </cols>
@@ -2024,2495 +1946,2495 @@
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
+      <c r="B1" s="4"/>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
+      <c r="B2" s="4"/>
     </row>
     <row r="3" ht="14.25" customHeight="1">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="7"/>
+      <c r="B3" s="5"/>
     </row>
     <row r="4" ht="28.5" customHeight="1">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="8" t="s">
+      <c r="B4" s="6"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="12" t="s">
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="13"/>
-      <c r="L4" s="14"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="12"/>
     </row>
     <row r="5" ht="14.25" customHeight="1">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="10" t="s">
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="11"/>
-      <c r="J5" s="12" t="s">
+      <c r="I5" s="9"/>
+      <c r="J5" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="K5" s="12" t="s">
+      <c r="K5" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="12" t="s">
+      <c r="L5" s="10" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8" t="s">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="13"/>
+      <c r="L6" s="13"/>
     </row>
     <row r="7" ht="6" customHeight="1">
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
     </row>
     <row r="8" ht="14.25" customHeight="1">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="17" t="s">
+      <c r="B8" s="14"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="13"/>
-      <c r="L8" s="14"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="12"/>
     </row>
     <row r="9" ht="6" customHeight="1">
       <c r="B9" s="1"/>
       <c r="D9"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
     </row>
     <row r="10" ht="14.25">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="20" t="s">
+      <c r="C10" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="D10" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="22" t="s">
+      <c r="E10" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="23" t="s">
+      <c r="F10" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G10" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="H10" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="J10" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="K10" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="L10" s="25" t="s">
+      <c r="G10" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J10" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K10" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="L10" s="22" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="11" ht="71.25" customHeight="1">
-      <c r="A11" s="26"/>
-      <c r="B11" s="27"/>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="29" t="s">
+      <c r="A11" s="23"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="30"/>
-      <c r="H11" s="26"/>
-      <c r="J11" s="31"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="26"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="23"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
     </row>
     <row r="12" ht="42.75" customHeight="1">
-      <c r="A12" s="26"/>
-      <c r="B12" s="32"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="29" t="s">
+      <c r="A12" s="23"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="30"/>
-      <c r="H12" s="26"/>
-      <c r="J12" s="31"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="26"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="23"/>
+      <c r="J12" s="28"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="23"/>
     </row>
     <row r="13" ht="57" customHeight="1">
-      <c r="A13" s="26"/>
-      <c r="B13" s="32"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="29" t="s">
+      <c r="A13" s="23"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="30"/>
-      <c r="H13" s="26"/>
-      <c r="J13" s="31"/>
-      <c r="K13" s="26"/>
-      <c r="L13" s="26"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="23"/>
+      <c r="J13" s="28"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="23"/>
     </row>
     <row r="14" ht="42.75" customHeight="1">
-      <c r="A14" s="26"/>
-      <c r="B14" s="32"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="29" t="s">
+      <c r="A14" s="23"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="30"/>
-      <c r="H14" s="26"/>
-      <c r="J14" s="31"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="26"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="23"/>
+      <c r="J14" s="28"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="23"/>
     </row>
     <row r="15" ht="28.5" customHeight="1">
-      <c r="A15" s="26"/>
-      <c r="B15" s="32"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="33" t="s">
+      <c r="A15" s="23"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="G15" s="30"/>
-      <c r="H15" s="26"/>
-      <c r="J15" s="34"/>
-      <c r="K15" s="26"/>
-      <c r="L15" s="26"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="23"/>
+      <c r="J15" s="31"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="23"/>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" s="35"/>
-      <c r="B16" s="36"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="38" t="s">
+      <c r="A16" s="32"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="39"/>
-      <c r="H16" s="35"/>
-      <c r="J16" s="40" t="s">
+      <c r="G16" s="36"/>
+      <c r="H16" s="32"/>
+      <c r="J16" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="K16" s="35"/>
-      <c r="L16" s="35"/>
+      <c r="K16" s="32"/>
+      <c r="L16" s="32"/>
     </row>
     <row r="17" ht="71.25" customHeight="1">
-      <c r="A17" s="41" t="s">
+      <c r="A17" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="42" t="s">
+      <c r="B17" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="43" t="s">
+      <c r="C17" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="41" t="s">
+      <c r="D17" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="E17" s="44" t="s">
+      <c r="E17" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="45" t="s">
+      <c r="F17" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="G17" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="H17" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="J17" s="47" t="s">
+      <c r="G17" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="H17" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="J17" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="K17" s="48" t="s">
+      <c r="K17" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="L17" s="49" t="s">
+      <c r="L17" s="44" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="18" ht="14.25">
-      <c r="A18" s="35"/>
-      <c r="B18" s="50"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="51" t="s">
+      <c r="A18" s="32"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="J18" s="51" t="s">
+      <c r="G18" s="32"/>
+      <c r="H18" s="32"/>
+      <c r="J18" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="K18" s="52"/>
-      <c r="L18" s="35"/>
+      <c r="K18" s="46"/>
+      <c r="L18" s="32"/>
     </row>
     <row r="19" ht="114">
-      <c r="A19" s="21">
+      <c r="A19" s="18">
         <v>2</v>
       </c>
-      <c r="B19" s="53" t="s">
+      <c r="B19" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D19" s="25" t="s">
+      <c r="D19" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="E19" s="54" t="s">
+      <c r="E19" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="55" t="s">
+      <c r="F19" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="G19" s="56" t="s">
+      <c r="G19" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="H19" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="J19" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="K19" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="L19" s="25" t="s">
+      <c r="H19" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J19" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="K19" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="L19" s="22" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="35"/>
-      <c r="B20" s="50"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="35"/>
-      <c r="E20" s="35"/>
-      <c r="F20" s="40" t="s">
+      <c r="A20" s="32"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="G20" s="40" t="s">
+      <c r="G20" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="H20" s="35"/>
-      <c r="J20" s="40" t="s">
+      <c r="H20" s="32"/>
+      <c r="J20" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="K20" s="40" t="s">
+      <c r="K20" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="L20" s="35"/>
+      <c r="L20" s="32"/>
     </row>
     <row r="21" ht="128.25">
-      <c r="A21" s="41">
+      <c r="A21" s="38">
         <v>2</v>
       </c>
-      <c r="B21" s="42" t="s">
+      <c r="B21" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="43" t="s">
+      <c r="C21" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="D21" s="46" t="s">
+      <c r="D21" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="E21" s="58" t="s">
+      <c r="E21" s="51" t="s">
         <v>42</v>
       </c>
-      <c r="F21" s="59" t="s">
+      <c r="F21" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="G21" s="60" t="s">
+      <c r="G21" s="53" t="s">
         <v>44</v>
       </c>
-      <c r="H21" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="J21" s="61" t="s">
+      <c r="H21" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="J21" s="54" t="s">
         <v>45</v>
       </c>
-      <c r="K21" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="L21" s="49" t="s">
+      <c r="K21" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="L21" s="44" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" ht="14.25">
-      <c r="A22" s="35"/>
-      <c r="B22" s="50"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="51" t="s">
+      <c r="A22" s="32"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="G22" s="51" t="s">
+      <c r="G22" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="H22" s="35"/>
-      <c r="J22" s="51" t="s">
+      <c r="H22" s="32"/>
+      <c r="J22" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="51" t="s">
+      <c r="K22" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="L22" s="35"/>
+      <c r="L22" s="32"/>
     </row>
     <row r="23" ht="99.75" customHeight="1">
-      <c r="A23" s="21">
+      <c r="A23" s="18">
         <v>3</v>
       </c>
-      <c r="B23" s="53" t="s">
+      <c r="B23" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="20" t="s">
+      <c r="C23" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D23" s="21" t="s">
+      <c r="D23" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E23" s="54" t="s">
+      <c r="E23" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="F23" s="55" t="s">
+      <c r="F23" s="48" t="s">
         <v>51</v>
       </c>
-      <c r="G23" s="55" t="s">
+      <c r="G23" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="H23" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="J23" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="K23" s="23" t="s">
+      <c r="H23" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J23" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="K23" s="56" t="s">
         <v>53</v>
       </c>
-      <c r="L23" s="25" t="s">
+      <c r="L23" s="22" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="24" ht="14.25">
-      <c r="A24" s="35"/>
-      <c r="B24" s="50"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="40" t="s">
+      <c r="A24" s="32"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="G24" s="40" t="s">
+      <c r="G24" s="37" t="s">
         <v>55</v>
       </c>
-      <c r="H24" s="35"/>
-      <c r="J24" s="40" t="s">
+      <c r="H24" s="32"/>
+      <c r="J24" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="K24" s="40" t="s">
+      <c r="K24" s="37" t="s">
         <v>55</v>
       </c>
-      <c r="L24" s="35"/>
+      <c r="L24" s="32"/>
     </row>
     <row r="25" ht="71.25" customHeight="1">
-      <c r="A25" s="63">
+      <c r="A25" s="57">
         <v>4</v>
       </c>
-      <c r="B25" s="64" t="s">
+      <c r="B25" s="58" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="65" t="s">
+      <c r="C25" s="57" t="s">
         <v>57</v>
       </c>
-      <c r="D25" s="63" t="s">
+      <c r="D25" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="E25" s="66" t="s">
+      <c r="E25" s="59" t="s">
         <v>58</v>
       </c>
-      <c r="F25" s="67" t="s">
+      <c r="F25" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="G25" s="67" t="s">
+      <c r="G25" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="H25" s="67" t="s">
+      <c r="H25" s="60" t="s">
         <v>59</v>
       </c>
-      <c r="J25" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="K25" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="L25" s="62" t="s">
+      <c r="J25" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="K25" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="L25" s="55" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="26" ht="14.25">
-      <c r="A26" s="35"/>
-      <c r="B26" s="50"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="35"/>
-      <c r="E26" s="35"/>
-      <c r="F26" s="40" t="s">
+      <c r="A26" s="32"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="G26" s="40" t="s">
+      <c r="G26" s="37" t="s">
         <v>55</v>
       </c>
-      <c r="H26" s="40" t="s">
+      <c r="H26" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="J26" s="40" t="s">
+      <c r="J26" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="K26" s="40" t="s">
+      <c r="K26" s="37" t="s">
         <v>55</v>
       </c>
-      <c r="L26" s="40" t="s">
+      <c r="L26" s="37" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="27" ht="128.25" customHeight="1">
-      <c r="A27" s="21">
+      <c r="A27" s="18">
         <v>4</v>
       </c>
-      <c r="B27" s="68" t="s">
+      <c r="B27" s="50" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="54" t="s">
+      <c r="C27" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="D27" s="21" t="s">
+      <c r="D27" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="E27" s="54" t="s">
+      <c r="E27" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="F27" s="55" t="s">
+      <c r="F27" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="G27" s="55" t="s">
+      <c r="G27" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="H27" s="55" t="s">
+      <c r="H27" s="48" t="s">
         <v>66</v>
       </c>
-      <c r="J27" s="23" t="s">
+      <c r="J27" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="K27" s="23" t="s">
+      <c r="K27" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="L27" s="57" t="s">
+      <c r="L27" s="50" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="28" ht="14.25">
-      <c r="A28" s="35"/>
-      <c r="B28" s="69"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="35"/>
-      <c r="E28" s="35"/>
-      <c r="F28" s="40" t="s">
+      <c r="A28" s="32"/>
+      <c r="B28" s="61"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="G28" s="40" t="s">
+      <c r="G28" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="H28" s="40" t="s">
+      <c r="H28" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="J28" s="40" t="s">
+      <c r="J28" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="K28" s="40" t="s">
+      <c r="K28" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="L28" s="40" t="s">
+      <c r="L28" s="37" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="29" ht="71.25" customHeight="1">
-      <c r="A29" s="63">
+      <c r="A29" s="57">
         <v>5</v>
       </c>
-      <c r="B29" s="64" t="s">
+      <c r="B29" s="58" t="s">
         <v>71</v>
       </c>
-      <c r="C29" s="65" t="s">
+      <c r="C29" s="57" t="s">
         <v>72</v>
       </c>
-      <c r="D29" s="63" t="s">
+      <c r="D29" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="E29" s="66" t="s">
+      <c r="E29" s="59" t="s">
         <v>50</v>
       </c>
-      <c r="F29" s="67" t="s">
+      <c r="F29" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="G29" s="67" t="s">
+      <c r="G29" s="60" t="s">
         <v>74</v>
       </c>
-      <c r="H29" s="67" t="s">
+      <c r="H29" s="60" t="s">
         <v>75</v>
       </c>
-      <c r="J29" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="K29" s="61" t="s">
+      <c r="J29" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="K29" s="54" t="s">
         <v>76</v>
       </c>
-      <c r="L29" s="61" t="s">
+      <c r="L29" s="54" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="30" ht="14.25">
-      <c r="A30" s="35"/>
-      <c r="B30" s="50"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="35"/>
-      <c r="F30" s="40" t="s">
+      <c r="A30" s="32"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="37" t="s">
         <v>78</v>
       </c>
-      <c r="G30" s="40" t="s">
+      <c r="G30" s="37" t="s">
         <v>79</v>
       </c>
-      <c r="H30" s="40" t="s">
+      <c r="H30" s="37" t="s">
         <v>80</v>
       </c>
-      <c r="J30" s="40" t="s">
+      <c r="J30" s="37" t="s">
         <v>78</v>
       </c>
-      <c r="K30" s="40" t="s">
+      <c r="K30" s="37" t="s">
         <v>79</v>
       </c>
-      <c r="L30" s="40" t="s">
+      <c r="L30" s="37" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="31" ht="42.75" customHeight="1">
-      <c r="A31" s="21">
+      <c r="A31" s="18">
         <v>5</v>
       </c>
-      <c r="B31" s="70" t="s">
+      <c r="B31" s="47" t="s">
         <v>81</v>
       </c>
-      <c r="C31" s="20" t="s">
+      <c r="C31" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="D31" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E31" s="54" t="s">
+      <c r="E31" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="F31" s="55" t="s">
+      <c r="F31" s="48" t="s">
         <v>84</v>
       </c>
-      <c r="G31" s="55" t="s">
+      <c r="G31" s="48" t="s">
         <v>85</v>
       </c>
-      <c r="H31" s="55" t="s">
+      <c r="H31" s="48" t="s">
         <v>85</v>
       </c>
-      <c r="J31" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="K31" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="L31" s="57" t="s">
+      <c r="J31" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="K31" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="L31" s="50" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="32" ht="14.25">
-      <c r="A32" s="35"/>
-      <c r="B32" s="50"/>
-      <c r="C32" s="35"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
-      <c r="F32" s="40" t="s">
+      <c r="A32" s="32"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="G32" s="40" t="s">
+      <c r="G32" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="H32" s="40" t="s">
+      <c r="H32" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="J32" s="40" t="s">
+      <c r="J32" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="K32" s="40" t="s">
+      <c r="K32" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="L32" s="40" t="s">
+      <c r="L32" s="37" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="33" ht="171" customHeight="1">
-      <c r="A33" s="63">
+      <c r="A33" s="57">
         <v>5</v>
       </c>
-      <c r="B33" s="64" t="s">
+      <c r="B33" s="58" t="s">
         <v>89</v>
       </c>
-      <c r="C33" s="65" t="s">
+      <c r="C33" s="57" t="s">
         <v>90</v>
       </c>
-      <c r="D33" s="63" t="s">
+      <c r="D33" s="57" t="s">
         <v>91</v>
       </c>
-      <c r="E33" s="66" t="s">
+      <c r="E33" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="F33" s="71" t="s">
+      <c r="F33" s="62" t="s">
         <v>93</v>
       </c>
-      <c r="G33" s="67" t="s">
+      <c r="G33" s="60" t="s">
         <v>94</v>
       </c>
-      <c r="H33" s="67" t="s">
+      <c r="H33" s="60" t="s">
         <v>95</v>
       </c>
-      <c r="J33" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="K33" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="L33" s="61" t="s">
+      <c r="J33" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="K33" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="L33" s="54" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="34" ht="14.25">
-      <c r="A34" s="35"/>
-      <c r="B34" s="50"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="35"/>
-      <c r="E34" s="35"/>
-      <c r="F34" s="40" t="s">
+      <c r="A34" s="32"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="32"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="37" t="s">
         <v>97</v>
       </c>
-      <c r="G34" s="40" t="s">
+      <c r="G34" s="37" t="s">
         <v>98</v>
       </c>
-      <c r="H34" s="40" t="s">
+      <c r="H34" s="37" t="s">
         <v>99</v>
       </c>
-      <c r="J34" s="40" t="s">
+      <c r="J34" s="37" t="s">
         <v>97</v>
       </c>
-      <c r="K34" s="40" t="s">
+      <c r="K34" s="37" t="s">
         <v>98</v>
       </c>
-      <c r="L34" s="40" t="s">
+      <c r="L34" s="37" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="35" ht="213.75" customHeight="1">
-      <c r="A35" s="21">
+      <c r="A35" s="18">
         <v>6</v>
       </c>
-      <c r="B35" s="70" t="s">
+      <c r="B35" s="47" t="s">
         <v>100</v>
       </c>
-      <c r="C35" s="20" t="s">
+      <c r="C35" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="D35" s="25" t="s">
+      <c r="D35" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="E35" s="54" t="s">
+      <c r="E35" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="F35" s="55" t="s">
+      <c r="F35" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="G35" s="55" t="s">
+      <c r="G35" s="48" t="s">
         <v>103</v>
       </c>
-      <c r="H35" s="55" t="s">
+      <c r="H35" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="J35" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="K35" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="L35" s="57" t="s">
+      <c r="J35" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="K35" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="L35" s="50" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="36" ht="14.25">
-      <c r="A36" s="35"/>
-      <c r="B36" s="50"/>
-      <c r="C36" s="35"/>
-      <c r="D36" s="35"/>
-      <c r="E36" s="35"/>
-      <c r="F36" s="40" t="s">
+      <c r="A36" s="32"/>
+      <c r="B36" s="7"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="37" t="s">
         <v>97</v>
       </c>
-      <c r="G36" s="40" t="s">
+      <c r="G36" s="37" t="s">
         <v>104</v>
       </c>
-      <c r="H36" s="40" t="s">
+      <c r="H36" s="37" t="s">
         <v>99</v>
       </c>
-      <c r="J36" s="40" t="s">
+      <c r="J36" s="37" t="s">
         <v>97</v>
       </c>
-      <c r="K36" s="40" t="s">
+      <c r="K36" s="37" t="s">
         <v>104</v>
       </c>
-      <c r="L36" s="40" t="s">
+      <c r="L36" s="37" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="37" ht="142.5" customHeight="1">
-      <c r="A37" s="63">
+      <c r="A37" s="57">
         <v>6</v>
       </c>
-      <c r="B37" s="64" t="s">
+      <c r="B37" s="58" t="s">
         <v>105</v>
       </c>
-      <c r="C37" s="65" t="s">
+      <c r="C37" s="57" t="s">
         <v>106</v>
       </c>
-      <c r="D37" s="72" t="s">
+      <c r="D37" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="E37" s="66" t="s">
+      <c r="E37" s="59" t="s">
         <v>107</v>
       </c>
-      <c r="F37" s="71" t="s">
+      <c r="F37" s="62" t="s">
         <v>108</v>
       </c>
-      <c r="G37" s="67" t="s">
+      <c r="G37" s="60" t="s">
         <v>109</v>
       </c>
-      <c r="H37" s="67" t="s">
+      <c r="H37" s="60" t="s">
         <v>110</v>
       </c>
-      <c r="J37" s="73" t="s">
+      <c r="J37" s="63" t="s">
         <v>111</v>
       </c>
-      <c r="K37" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="L37" s="61" t="s">
+      <c r="K37" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="L37" s="54" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="38" ht="14.25">
-      <c r="A38" s="35"/>
-      <c r="B38" s="50"/>
-      <c r="C38" s="35"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="35"/>
-      <c r="F38" s="40" t="s">
+      <c r="A38" s="32"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="37" t="s">
         <v>113</v>
       </c>
-      <c r="G38" s="40" t="s">
+      <c r="G38" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="H38" s="40" t="s">
+      <c r="H38" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="J38" s="40" t="s">
+      <c r="J38" s="37" t="s">
         <v>113</v>
       </c>
-      <c r="K38" s="40" t="s">
+      <c r="K38" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="L38" s="40" t="s">
+      <c r="L38" s="37" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="39" ht="57" customHeight="1">
-      <c r="A39" s="74">
+      <c r="A39" s="64">
         <v>6</v>
       </c>
-      <c r="B39" s="75" t="s">
+      <c r="B39" s="64" t="s">
         <v>116</v>
       </c>
-      <c r="C39" s="76" t="s">
+      <c r="C39" s="64" t="s">
         <v>117</v>
       </c>
-      <c r="D39" s="77" t="s">
+      <c r="D39" s="65" t="s">
         <v>10</v>
       </c>
-      <c r="E39" s="78" t="s">
+      <c r="E39" s="65" t="s">
         <v>118</v>
       </c>
-      <c r="F39" s="55" t="s">
+      <c r="F39" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="G39" s="79" t="s">
+      <c r="G39" s="66" t="s">
         <v>119</v>
       </c>
-      <c r="H39" s="55" t="s">
+      <c r="H39" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="J39" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="K39" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="L39" s="57" t="s">
+      <c r="J39" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="K39" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="L39" s="50" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="40" ht="14.25">
-      <c r="A40" s="26"/>
-      <c r="B40" s="80"/>
-      <c r="C40" s="26"/>
-      <c r="D40" s="26"/>
-      <c r="E40" s="26"/>
-      <c r="F40" s="40" t="s">
+      <c r="A40" s="23"/>
+      <c r="B40" s="23"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="23"/>
+      <c r="E40" s="23"/>
+      <c r="F40" s="37" t="s">
         <v>113</v>
       </c>
-      <c r="G40" s="40" t="s">
+      <c r="G40" s="37" t="s">
         <v>120</v>
       </c>
-      <c r="H40" s="40" t="s">
+      <c r="H40" s="37" t="s">
         <v>115</v>
       </c>
-      <c r="J40" s="40" t="s">
+      <c r="J40" s="37" t="s">
         <v>113</v>
       </c>
-      <c r="K40" s="40" t="s">
+      <c r="K40" s="37" t="s">
         <v>120</v>
       </c>
-      <c r="L40" s="40" t="s">
+      <c r="L40" s="37" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="41" ht="99.75" customHeight="1">
-      <c r="A41" s="63">
+      <c r="A41" s="57">
         <v>7</v>
       </c>
-      <c r="B41" s="64" t="s">
+      <c r="B41" s="58" t="s">
         <v>121</v>
       </c>
-      <c r="C41" s="65" t="s">
+      <c r="C41" s="57" t="s">
         <v>122</v>
       </c>
-      <c r="D41" s="63" t="s">
+      <c r="D41" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="E41" s="66" t="s">
+      <c r="E41" s="59" t="s">
         <v>123</v>
       </c>
-      <c r="F41" s="71" t="s">
+      <c r="F41" s="62" t="s">
         <v>124</v>
       </c>
-      <c r="G41" s="71" t="s">
+      <c r="G41" s="62" t="s">
         <v>125</v>
       </c>
-      <c r="H41" s="67" t="s">
+      <c r="H41" s="60" t="s">
         <v>126</v>
       </c>
-      <c r="J41" s="73" t="s">
+      <c r="J41" s="63" t="s">
         <v>127</v>
       </c>
-      <c r="K41" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="L41" s="62" t="s">
+      <c r="K41" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="L41" s="55" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="42" ht="14.25" customHeight="1">
-      <c r="A42" s="35"/>
-      <c r="B42" s="50"/>
-      <c r="C42" s="35"/>
-      <c r="D42" s="35"/>
-      <c r="E42" s="35"/>
-      <c r="F42" s="40" t="s">
+      <c r="A42" s="32"/>
+      <c r="B42" s="7"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="G42" s="40" t="s">
+      <c r="G42" s="37" t="s">
         <v>129</v>
       </c>
-      <c r="H42" s="40" t="s">
+      <c r="H42" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="J42" s="40" t="s">
+      <c r="J42" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="K42" s="40" t="s">
+      <c r="K42" s="37" t="s">
         <v>129</v>
       </c>
-      <c r="L42" s="40" t="s">
+      <c r="L42" s="37" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="43" ht="6" customHeight="1">
-      <c r="C43" s="81"/>
-      <c r="D43" s="81"/>
-      <c r="E43" s="81"/>
-      <c r="F43" s="81"/>
-      <c r="G43" s="81"/>
-      <c r="H43" s="81"/>
-      <c r="I43" s="81"/>
+      <c r="C43" s="67"/>
+      <c r="D43" s="67"/>
+      <c r="E43" s="67"/>
+      <c r="F43" s="67"/>
+      <c r="G43" s="67"/>
+      <c r="H43" s="67"/>
+      <c r="I43" s="67"/>
     </row>
     <row r="44" ht="14.25" customHeight="1">
-      <c r="A44" s="8" t="s">
+      <c r="A44" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="B44" s="16"/>
-      <c r="C44" s="13"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
-      <c r="F44" s="13"/>
-      <c r="G44" s="13"/>
-      <c r="H44" s="14"/>
-      <c r="J44" s="17" t="s">
+      <c r="B44" s="14"/>
+      <c r="C44" s="11"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="11"/>
+      <c r="G44" s="11"/>
+      <c r="H44" s="12"/>
+      <c r="J44" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="K44" s="13"/>
-      <c r="L44" s="14"/>
+      <c r="K44" s="11"/>
+      <c r="L44" s="12"/>
     </row>
     <row r="45" ht="6" customHeight="1">
       <c r="A45" s="1"/>
-      <c r="B45" s="82"/>
+      <c r="B45" s="1"/>
       <c r="D45"/>
       <c r="E45" s="3"/>
     </row>
     <row r="46" ht="14.25" customHeight="1">
-      <c r="A46" s="21" t="s">
+      <c r="A46" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B46" s="70" t="s">
+      <c r="B46" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="C46" s="20" t="s">
+      <c r="C46" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D46" s="21" t="s">
+      <c r="D46" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E46" s="22" t="s">
+      <c r="E46" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="F46" s="23" t="s">
+      <c r="F46" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="G46" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="H46" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="J46" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="K46" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="L46" s="25" t="s">
+      <c r="G46" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="H46" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J46" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K46" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="L46" s="22" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="47" ht="28.5" customHeight="1">
-      <c r="A47" s="26"/>
-      <c r="B47" s="83"/>
-      <c r="C47" s="26"/>
-      <c r="D47" s="26"/>
-      <c r="E47" s="28"/>
-      <c r="F47" s="29" t="s">
+      <c r="A47" s="23"/>
+      <c r="B47" s="68"/>
+      <c r="C47" s="23"/>
+      <c r="D47" s="23"/>
+      <c r="E47" s="25"/>
+      <c r="F47" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="G47" s="30"/>
-      <c r="H47" s="26"/>
-      <c r="J47" s="31"/>
-      <c r="K47" s="26"/>
-      <c r="L47" s="26"/>
+      <c r="G47" s="27"/>
+      <c r="H47" s="23"/>
+      <c r="J47" s="28"/>
+      <c r="K47" s="23"/>
+      <c r="L47" s="23"/>
     </row>
     <row r="48" ht="28.5" customHeight="1">
-      <c r="A48" s="26"/>
-      <c r="B48" s="84"/>
-      <c r="C48" s="26"/>
-      <c r="D48" s="26"/>
-      <c r="E48" s="28"/>
-      <c r="F48" s="29" t="s">
+      <c r="A48" s="23"/>
+      <c r="B48" s="23"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="23"/>
+      <c r="E48" s="25"/>
+      <c r="F48" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="G48" s="30"/>
-      <c r="H48" s="26"/>
-      <c r="J48" s="31"/>
-      <c r="K48" s="26"/>
-      <c r="L48" s="26"/>
+      <c r="G48" s="27"/>
+      <c r="H48" s="23"/>
+      <c r="J48" s="28"/>
+      <c r="K48" s="23"/>
+      <c r="L48" s="23"/>
     </row>
     <row r="49" ht="85.5" customHeight="1">
-      <c r="A49" s="26"/>
-      <c r="B49" s="84"/>
-      <c r="C49" s="26"/>
-      <c r="D49" s="26"/>
-      <c r="E49" s="28"/>
-      <c r="F49" s="29" t="s">
+      <c r="A49" s="23"/>
+      <c r="B49" s="23"/>
+      <c r="C49" s="23"/>
+      <c r="D49" s="23"/>
+      <c r="E49" s="25"/>
+      <c r="F49" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="G49" s="30"/>
-      <c r="H49" s="26"/>
-      <c r="J49" s="31"/>
-      <c r="K49" s="26"/>
-      <c r="L49" s="26"/>
+      <c r="G49" s="27"/>
+      <c r="H49" s="23"/>
+      <c r="J49" s="28"/>
+      <c r="K49" s="23"/>
+      <c r="L49" s="23"/>
     </row>
     <row r="50" ht="57" customHeight="1">
-      <c r="A50" s="26"/>
-      <c r="B50" s="84"/>
-      <c r="C50" s="26"/>
-      <c r="D50" s="26"/>
-      <c r="E50" s="28"/>
-      <c r="F50" s="29" t="s">
+      <c r="A50" s="23"/>
+      <c r="B50" s="23"/>
+      <c r="C50" s="23"/>
+      <c r="D50" s="23"/>
+      <c r="E50" s="25"/>
+      <c r="F50" s="69" t="s">
         <v>136</v>
       </c>
-      <c r="G50" s="30"/>
-      <c r="H50" s="26"/>
-      <c r="J50" s="31"/>
-      <c r="K50" s="26"/>
-      <c r="L50" s="26"/>
+      <c r="G50" s="27"/>
+      <c r="H50" s="23"/>
+      <c r="J50" s="28"/>
+      <c r="K50" s="23"/>
+      <c r="L50" s="23"/>
     </row>
     <row r="51" ht="42.75" customHeight="1">
-      <c r="A51" s="26"/>
-      <c r="B51" s="84"/>
-      <c r="C51" s="26"/>
-      <c r="D51" s="26"/>
-      <c r="E51" s="28"/>
-      <c r="F51" s="29" t="s">
+      <c r="A51" s="23"/>
+      <c r="B51" s="23"/>
+      <c r="C51" s="23"/>
+      <c r="D51" s="23"/>
+      <c r="E51" s="25"/>
+      <c r="F51" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="G51" s="30"/>
-      <c r="H51" s="26"/>
-      <c r="J51" s="31"/>
-      <c r="K51" s="26"/>
-      <c r="L51" s="26"/>
+      <c r="G51" s="27"/>
+      <c r="H51" s="23"/>
+      <c r="J51" s="28"/>
+      <c r="K51" s="23"/>
+      <c r="L51" s="23"/>
     </row>
     <row r="52" ht="57" customHeight="1">
-      <c r="A52" s="26"/>
-      <c r="B52" s="84"/>
-      <c r="C52" s="26"/>
-      <c r="D52" s="26"/>
-      <c r="E52" s="28"/>
-      <c r="F52" s="33" t="s">
+      <c r="A52" s="23"/>
+      <c r="B52" s="23"/>
+      <c r="C52" s="23"/>
+      <c r="D52" s="23"/>
+      <c r="E52" s="25"/>
+      <c r="F52" s="30" t="s">
         <v>138</v>
       </c>
-      <c r="G52" s="30"/>
-      <c r="H52" s="26"/>
-      <c r="J52" s="34"/>
-      <c r="K52" s="26"/>
-      <c r="L52" s="26"/>
+      <c r="G52" s="27"/>
+      <c r="H52" s="23"/>
+      <c r="J52" s="31"/>
+      <c r="K52" s="23"/>
+      <c r="L52" s="23"/>
     </row>
     <row r="53" ht="14.25" customHeight="1">
-      <c r="A53" s="35"/>
-      <c r="B53" s="85"/>
-      <c r="C53" s="35"/>
-      <c r="D53" s="35"/>
-      <c r="E53" s="35"/>
-      <c r="F53" s="38" t="s">
+      <c r="A53" s="32"/>
+      <c r="B53" s="32"/>
+      <c r="C53" s="32"/>
+      <c r="D53" s="32"/>
+      <c r="E53" s="32"/>
+      <c r="F53" s="70" t="s">
         <v>139</v>
       </c>
-      <c r="G53" s="35"/>
-      <c r="H53" s="35"/>
-      <c r="J53" s="40" t="s">
-        <v>139</v>
-      </c>
-      <c r="K53" s="35"/>
-      <c r="L53" s="35"/>
+      <c r="G53" s="32"/>
+      <c r="H53" s="32"/>
+      <c r="J53" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="K53" s="32"/>
+      <c r="L53" s="32"/>
     </row>
     <row r="54" ht="57" customHeight="1">
-      <c r="A54" s="41" t="s">
+      <c r="A54" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="B54" s="86" t="s">
+      <c r="B54" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="C54" s="43" t="s">
+      <c r="C54" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="D54" s="41" t="s">
+      <c r="D54" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="E54" s="44" t="s">
-        <v>140</v>
-      </c>
-      <c r="F54" s="45" t="s">
+      <c r="E54" s="40" t="s">
         <v>141</v>
       </c>
-      <c r="G54" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="H54" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="J54" s="47" t="s">
+      <c r="F54" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="K54" s="49" t="s">
-        <v>20</v>
-      </c>
-      <c r="L54" s="49" t="s">
+      <c r="G54" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="H54" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="J54" s="42" t="s">
+        <v>143</v>
+      </c>
+      <c r="K54" s="44" t="s">
+        <v>20</v>
+      </c>
+      <c r="L54" s="44" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="55" ht="14.25" customHeight="1">
-      <c r="A55" s="35"/>
-      <c r="B55" s="50"/>
-      <c r="C55" s="35"/>
-      <c r="D55" s="35"/>
-      <c r="E55" s="35"/>
-      <c r="F55" s="51" t="s">
-        <v>143</v>
-      </c>
-      <c r="G55" s="35"/>
-      <c r="H55" s="35"/>
-      <c r="J55" s="51" t="s">
-        <v>143</v>
-      </c>
-      <c r="K55" s="35"/>
-      <c r="L55" s="35"/>
+      <c r="A55" s="32"/>
+      <c r="B55" s="7"/>
+      <c r="C55" s="32"/>
+      <c r="D55" s="32"/>
+      <c r="E55" s="32"/>
+      <c r="F55" s="45" t="s">
+        <v>144</v>
+      </c>
+      <c r="G55" s="32"/>
+      <c r="H55" s="32"/>
+      <c r="J55" s="45" t="s">
+        <v>144</v>
+      </c>
+      <c r="K55" s="32"/>
+      <c r="L55" s="32"/>
     </row>
     <row r="56" ht="57" customHeight="1">
-      <c r="A56" s="21">
+      <c r="A56" s="18">
         <v>1</v>
       </c>
-      <c r="B56" s="70" t="s">
-        <v>144</v>
-      </c>
-      <c r="C56" s="20" t="s">
+      <c r="B56" s="47" t="s">
         <v>145</v>
       </c>
-      <c r="D56" s="25" t="s">
+      <c r="C56" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="D56" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="E56" s="54" t="s">
-        <v>146</v>
-      </c>
-      <c r="F56" s="55" t="s">
+      <c r="E56" s="22" t="s">
         <v>147</v>
       </c>
-      <c r="G56" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="H56" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="J56" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="K56" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="L56" s="25" t="s">
+      <c r="F56" s="72" t="s">
+        <v>148</v>
+      </c>
+      <c r="G56" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="H56" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J56" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="K56" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="L56" s="22" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="57" ht="14.25" customHeight="1">
-      <c r="A57" s="35"/>
-      <c r="B57" s="50"/>
-      <c r="C57" s="35"/>
-      <c r="D57" s="35"/>
-      <c r="E57" s="35"/>
-      <c r="F57" s="40" t="s">
-        <v>148</v>
-      </c>
-      <c r="G57" s="35"/>
-      <c r="H57" s="35"/>
-      <c r="J57" s="40" t="s">
-        <v>148</v>
-      </c>
-      <c r="K57" s="35"/>
-      <c r="L57" s="35"/>
+      <c r="A57" s="32"/>
+      <c r="B57" s="7"/>
+      <c r="C57" s="32"/>
+      <c r="D57" s="32"/>
+      <c r="E57" s="32"/>
+      <c r="F57" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="G57" s="32"/>
+      <c r="H57" s="32"/>
+      <c r="J57" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="K57" s="32"/>
+      <c r="L57" s="32"/>
     </row>
     <row r="58" ht="71.25" customHeight="1">
-      <c r="A58" s="63">
+      <c r="A58" s="57">
         <v>4</v>
       </c>
-      <c r="B58" s="64" t="s">
+      <c r="B58" s="58" t="s">
         <v>56</v>
       </c>
-      <c r="C58" s="65" t="s">
+      <c r="C58" s="57" t="s">
         <v>57</v>
       </c>
-      <c r="D58" s="63" t="s">
+      <c r="D58" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="E58" s="66" t="s">
+      <c r="E58" s="59" t="s">
         <v>58</v>
       </c>
-      <c r="F58" s="87" t="s">
+      <c r="F58" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="G58" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="H58" s="67" t="s">
+      <c r="G58" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="H58" s="60" t="s">
         <v>59</v>
       </c>
-      <c r="J58" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="K58" s="49" t="s">
-        <v>20</v>
-      </c>
-      <c r="L58" s="62" t="s">
+      <c r="J58" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="K58" s="44" t="s">
+        <v>20</v>
+      </c>
+      <c r="L58" s="55" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="59" ht="14.25" customHeight="1">
-      <c r="A59" s="35"/>
-      <c r="B59" s="50"/>
-      <c r="C59" s="35"/>
-      <c r="D59" s="35"/>
-      <c r="E59" s="35"/>
-      <c r="F59" s="40" t="s">
-        <v>148</v>
-      </c>
-      <c r="G59" s="35"/>
-      <c r="H59" s="38" t="s">
+      <c r="A59" s="32"/>
+      <c r="B59" s="7"/>
+      <c r="C59" s="32"/>
+      <c r="D59" s="32"/>
+      <c r="E59" s="32"/>
+      <c r="F59" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="G59" s="32"/>
+      <c r="H59" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="J59" s="40" t="s">
-        <v>148</v>
-      </c>
-      <c r="K59" s="35"/>
-      <c r="L59" s="40" t="s">
+      <c r="J59" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="K59" s="32"/>
+      <c r="L59" s="37" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="60" ht="128.25" customHeight="1">
-      <c r="A60" s="21">
+      <c r="A60" s="18">
         <v>4</v>
       </c>
-      <c r="B60" s="70" t="s">
+      <c r="B60" s="47" t="s">
         <v>61</v>
       </c>
-      <c r="C60" s="20" t="s">
+      <c r="C60" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="D60" s="25" t="s">
+      <c r="D60" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="E60" s="54" t="s">
+      <c r="E60" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="F60" s="55" t="s">
+      <c r="F60" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="G60" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="H60" s="55" t="s">
+      <c r="G60" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="H60" s="48" t="s">
         <v>66</v>
       </c>
-      <c r="J60" s="88" t="s">
-        <v>149</v>
-      </c>
-      <c r="K60" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="L60" s="57" t="s">
+      <c r="J60" s="74" t="s">
+        <v>150</v>
+      </c>
+      <c r="K60" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="L60" s="50" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="61" ht="14.25" customHeight="1">
-      <c r="A61" s="35"/>
-      <c r="B61" s="50"/>
-      <c r="C61" s="35"/>
-      <c r="D61" s="35"/>
-      <c r="E61" s="35"/>
-      <c r="F61" s="40" t="s">
+      <c r="A61" s="32"/>
+      <c r="B61" s="7"/>
+      <c r="C61" s="32"/>
+      <c r="D61" s="32"/>
+      <c r="E61" s="32"/>
+      <c r="F61" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="G61" s="35"/>
-      <c r="H61" s="38" t="s">
+      <c r="G61" s="32"/>
+      <c r="H61" s="35" t="s">
         <v>70</v>
       </c>
-      <c r="J61" s="40" t="s">
+      <c r="J61" s="37" t="s">
         <v>68</v>
       </c>
-      <c r="K61" s="35"/>
-      <c r="L61" s="40" t="s">
+      <c r="K61" s="32"/>
+      <c r="L61" s="37" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="62" ht="42.75" customHeight="1">
-      <c r="A62" s="63">
+      <c r="A62" s="57">
         <v>5</v>
       </c>
-      <c r="B62" s="64" t="s">
+      <c r="B62" s="58" t="s">
         <v>71</v>
       </c>
-      <c r="C62" s="65" t="s">
+      <c r="C62" s="57" t="s">
         <v>72</v>
       </c>
-      <c r="D62" s="63" t="s">
+      <c r="D62" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="E62" s="66" t="s">
+      <c r="E62" s="59" t="s">
         <v>50</v>
       </c>
-      <c r="F62" s="67" t="s">
+      <c r="F62" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="G62" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="H62" s="67" t="s">
+      <c r="G62" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="H62" s="60" t="s">
         <v>75</v>
       </c>
-      <c r="J62" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="K62" s="49" t="s">
-        <v>20</v>
-      </c>
-      <c r="L62" s="89" t="s">
-        <v>150</v>
+      <c r="J62" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="K62" s="44" t="s">
+        <v>20</v>
+      </c>
+      <c r="L62" s="75" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
-      <c r="A63" s="35"/>
-      <c r="B63" s="50"/>
-      <c r="C63" s="35"/>
-      <c r="D63" s="35"/>
-      <c r="E63" s="35"/>
-      <c r="F63" s="40" t="s">
+      <c r="A63" s="32"/>
+      <c r="B63" s="7"/>
+      <c r="C63" s="32"/>
+      <c r="D63" s="32"/>
+      <c r="E63" s="32"/>
+      <c r="F63" s="37" t="s">
         <v>78</v>
       </c>
-      <c r="G63" s="35"/>
-      <c r="H63" s="40" t="s">
+      <c r="G63" s="32"/>
+      <c r="H63" s="37" t="s">
         <v>80</v>
       </c>
-      <c r="J63" s="40" t="s">
+      <c r="J63" s="37" t="s">
         <v>78</v>
       </c>
-      <c r="K63" s="35"/>
-      <c r="L63" s="40" t="s">
+      <c r="K63" s="32"/>
+      <c r="L63" s="37" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="64" ht="42.75" customHeight="1">
-      <c r="A64" s="21">
+      <c r="A64" s="18">
         <v>5</v>
       </c>
-      <c r="B64" s="70" t="s">
+      <c r="B64" s="47" t="s">
         <v>81</v>
       </c>
-      <c r="C64" s="20" t="s">
+      <c r="C64" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="D64" s="21" t="s">
+      <c r="D64" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E64" s="54" t="s">
+      <c r="E64" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="F64" s="55" t="s">
+      <c r="F64" s="48" t="s">
         <v>84</v>
       </c>
-      <c r="G64" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="H64" s="55" t="s">
+      <c r="G64" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="H64" s="48" t="s">
         <v>85</v>
       </c>
-      <c r="J64" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="K64" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="L64" s="57" t="s">
+      <c r="J64" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="K64" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="L64" s="50" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="65" ht="14.25" customHeight="1">
-      <c r="A65" s="35"/>
-      <c r="B65" s="50"/>
-      <c r="C65" s="35"/>
-      <c r="D65" s="35"/>
-      <c r="E65" s="35"/>
-      <c r="F65" s="40" t="s">
+      <c r="A65" s="32"/>
+      <c r="B65" s="7"/>
+      <c r="C65" s="32"/>
+      <c r="D65" s="32"/>
+      <c r="E65" s="32"/>
+      <c r="F65" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="G65" s="35"/>
-      <c r="H65" s="40" t="s">
+      <c r="G65" s="32"/>
+      <c r="H65" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="J65" s="40" t="s">
+      <c r="J65" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="K65" s="35"/>
-      <c r="L65" s="40" t="s">
+      <c r="K65" s="32"/>
+      <c r="L65" s="37" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="66" ht="14.25" customHeight="1">
-      <c r="A66" s="63">
+      <c r="A66" s="57">
         <v>5</v>
       </c>
-      <c r="B66" s="64" t="s">
+      <c r="B66" s="58" t="s">
         <v>89</v>
       </c>
-      <c r="C66" s="65" t="s">
+      <c r="C66" s="57" t="s">
         <v>90</v>
       </c>
-      <c r="D66" s="63" t="s">
+      <c r="D66" s="57" t="s">
         <v>91</v>
       </c>
-      <c r="E66" s="66" t="s">
+      <c r="E66" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="F66" s="71" t="s">
-        <v>151</v>
-      </c>
-      <c r="G66" s="46" t="s">
-        <v>20</v>
-      </c>
-      <c r="H66" s="67" t="s">
+      <c r="F66" s="62" t="s">
         <v>152</v>
       </c>
-      <c r="J66" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="K66" s="49" t="s">
-        <v>20</v>
-      </c>
-      <c r="L66" s="61" t="s">
+      <c r="G66" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="H66" s="60" t="s">
         <v>153</v>
       </c>
+      <c r="J66" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="K66" s="44" t="s">
+        <v>20</v>
+      </c>
+      <c r="L66" s="54" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="67" ht="14.25" customHeight="1">
-      <c r="A67" s="35"/>
-      <c r="B67" s="50"/>
-      <c r="C67" s="35"/>
-      <c r="D67" s="35"/>
-      <c r="E67" s="35"/>
-      <c r="F67" s="40" t="s">
-        <v>154</v>
-      </c>
-      <c r="G67" s="35"/>
-      <c r="H67" s="40" t="s">
+      <c r="A67" s="32"/>
+      <c r="B67" s="7"/>
+      <c r="C67" s="32"/>
+      <c r="D67" s="32"/>
+      <c r="E67" s="32"/>
+      <c r="F67" s="37" t="s">
         <v>155</v>
       </c>
-      <c r="J67" s="40" t="s">
-        <v>154</v>
-      </c>
-      <c r="K67" s="35"/>
-      <c r="L67" s="40" t="s">
+      <c r="G67" s="32"/>
+      <c r="H67" s="37" t="s">
+        <v>156</v>
+      </c>
+      <c r="J67" s="37" t="s">
         <v>155</v>
       </c>
+      <c r="K67" s="32"/>
+      <c r="L67" s="37" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="68" ht="14.25" customHeight="1">
-      <c r="A68" s="21">
+      <c r="A68" s="18">
         <v>7</v>
       </c>
-      <c r="B68" s="70" t="s">
+      <c r="B68" s="47" t="s">
         <v>121</v>
       </c>
-      <c r="C68" s="20" t="s">
+      <c r="C68" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="D68" s="21" t="s">
+      <c r="D68" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="E68" s="54" t="s">
+      <c r="E68" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="F68" s="90" t="s">
+      <c r="F68" s="76" t="s">
         <v>124</v>
       </c>
-      <c r="G68" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="H68" s="55" t="s">
+      <c r="G68" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="H68" s="48" t="s">
         <v>126</v>
       </c>
-      <c r="J68" s="88" t="s">
-        <v>156</v>
-      </c>
-      <c r="K68" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="L68" s="91" t="s">
+      <c r="J68" s="74" t="s">
+        <v>157</v>
+      </c>
+      <c r="K68" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="L68" s="77" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="69" ht="14.25" customHeight="1">
-      <c r="A69" s="35"/>
-      <c r="B69" s="50"/>
-      <c r="C69" s="35"/>
-      <c r="D69" s="35"/>
-      <c r="E69" s="35"/>
-      <c r="F69" s="40" t="s">
+      <c r="A69" s="32"/>
+      <c r="B69" s="7"/>
+      <c r="C69" s="32"/>
+      <c r="D69" s="32"/>
+      <c r="E69" s="32"/>
+      <c r="F69" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="G69" s="35"/>
-      <c r="H69" s="40" t="s">
+      <c r="G69" s="32"/>
+      <c r="H69" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="J69" s="40" t="s">
+      <c r="J69" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="K69" s="35"/>
-      <c r="L69" s="40" t="s">
+      <c r="K69" s="32"/>
+      <c r="L69" s="37" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="70" ht="14.25" customHeight="1"/>
     <row r="71" ht="14.25" customHeight="1">
-      <c r="A71" s="92" t="s">
-        <v>157</v>
-      </c>
-      <c r="B71" s="93"/>
-      <c r="C71" s="13"/>
-      <c r="D71" s="13"/>
-      <c r="E71" s="13"/>
-      <c r="F71" s="13"/>
-      <c r="G71" s="13"/>
-      <c r="H71" s="14"/>
-      <c r="J71" s="12" t="s">
-        <v>157</v>
-      </c>
-      <c r="K71" s="13"/>
-      <c r="L71" s="14"/>
+      <c r="A71" s="78" t="s">
+        <v>158</v>
+      </c>
+      <c r="B71" s="79"/>
+      <c r="C71" s="11"/>
+      <c r="D71" s="11"/>
+      <c r="E71" s="11"/>
+      <c r="F71" s="11"/>
+      <c r="G71" s="11"/>
+      <c r="H71" s="12"/>
+      <c r="J71" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="K71" s="11"/>
+      <c r="L71" s="12"/>
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="D72"/>
     </row>
     <row r="73" ht="71.25" customHeight="1">
-      <c r="A73" s="21">
+      <c r="A73" s="18">
         <v>8</v>
       </c>
-      <c r="B73" s="70" t="s">
-        <v>158</v>
-      </c>
-      <c r="C73" s="20" t="s">
+      <c r="B73" s="47" t="s">
         <v>159</v>
       </c>
-      <c r="D73" s="21" t="s">
+      <c r="C73" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="D73" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="E73" s="54" t="s">
-        <v>160</v>
-      </c>
-      <c r="F73" s="55" t="s">
+      <c r="E73" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="F73" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="G73" s="55" t="s">
+      <c r="G73" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="H73" s="55" t="s">
-        <v>161</v>
-      </c>
-      <c r="J73" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="K73" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="L73" s="57" t="s">
+      <c r="H73" s="48" t="s">
+        <v>162</v>
+      </c>
+      <c r="J73" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="K73" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="L73" s="50" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="74" ht="14.25">
-      <c r="A74" s="35"/>
-      <c r="B74" s="50"/>
-      <c r="C74" s="35"/>
-      <c r="D74" s="35"/>
-      <c r="E74" s="35"/>
-      <c r="F74" s="40" t="s">
+      <c r="A74" s="32"/>
+      <c r="B74" s="7"/>
+      <c r="C74" s="32"/>
+      <c r="D74" s="32"/>
+      <c r="E74" s="32"/>
+      <c r="F74" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="G74" s="40" t="s">
+      <c r="G74" s="37" t="s">
         <v>129</v>
       </c>
-      <c r="H74" s="40" t="s">
-        <v>162</v>
-      </c>
-      <c r="J74" s="40" t="s">
+      <c r="H74" s="37" t="s">
+        <v>163</v>
+      </c>
+      <c r="J74" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="K74" s="40" t="s">
+      <c r="K74" s="37" t="s">
         <v>129</v>
       </c>
-      <c r="L74" s="40" t="s">
-        <v>162</v>
+      <c r="L74" s="37" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="75" ht="71.25" customHeight="1">
-      <c r="A75" s="63">
+      <c r="A75" s="57">
         <v>8</v>
       </c>
-      <c r="B75" s="64" t="s">
-        <v>163</v>
-      </c>
-      <c r="C75" s="65" t="s">
+      <c r="B75" s="58" t="s">
         <v>164</v>
       </c>
-      <c r="D75" s="63" t="s">
+      <c r="C75" s="57" t="s">
+        <v>165</v>
+      </c>
+      <c r="D75" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="E75" s="66" t="s">
-        <v>165</v>
-      </c>
-      <c r="F75" s="71" t="s">
+      <c r="E75" s="59" t="s">
         <v>166</v>
       </c>
-      <c r="G75" s="71" t="s">
+      <c r="F75" s="62" t="s">
         <v>167</v>
       </c>
-      <c r="H75" s="71" t="s">
+      <c r="G75" s="62" t="s">
         <v>168</v>
       </c>
-      <c r="J75" s="73" t="s">
+      <c r="H75" s="62" t="s">
         <v>169</v>
       </c>
-      <c r="K75" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="L75" s="62" t="s">
+      <c r="J75" s="63" t="s">
+        <v>170</v>
+      </c>
+      <c r="K75" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="L75" s="55" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="76" ht="14.25">
-      <c r="A76" s="35"/>
-      <c r="B76" s="50"/>
-      <c r="C76" s="35"/>
-      <c r="D76" s="35"/>
-      <c r="E76" s="35"/>
-      <c r="F76" s="40" t="s">
-        <v>170</v>
-      </c>
-      <c r="G76" s="40" t="s">
+      <c r="A76" s="32"/>
+      <c r="B76" s="7"/>
+      <c r="C76" s="32"/>
+      <c r="D76" s="32"/>
+      <c r="E76" s="32"/>
+      <c r="F76" s="37" t="s">
         <v>171</v>
       </c>
-      <c r="H76" s="40" t="s">
+      <c r="G76" s="37" t="s">
         <v>172</v>
       </c>
-      <c r="J76" s="40" t="s">
-        <v>170</v>
-      </c>
-      <c r="K76" s="40" t="s">
+      <c r="H76" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="J76" s="37" t="s">
         <v>171</v>
       </c>
-      <c r="L76" s="40" t="s">
+      <c r="K76" s="37" t="s">
         <v>172</v>
       </c>
+      <c r="L76" s="37" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="77" ht="71.25" customHeight="1">
-      <c r="A77" s="21">
+      <c r="A77" s="18">
         <v>9</v>
       </c>
-      <c r="B77" s="70" t="s">
-        <v>173</v>
-      </c>
-      <c r="C77" s="20" t="s">
+      <c r="B77" s="47" t="s">
         <v>174</v>
       </c>
-      <c r="D77" s="21" t="s">
+      <c r="C77" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="D77" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E77" s="54" t="s">
+      <c r="E77" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="F77" s="90" t="s">
-        <v>175</v>
-      </c>
-      <c r="G77" s="90" t="s">
+      <c r="F77" s="76" t="s">
         <v>176</v>
       </c>
-      <c r="H77" s="90" t="s">
+      <c r="G77" s="76" t="s">
         <v>177</v>
       </c>
-      <c r="J77" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="K77" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="L77" s="57" t="s">
+      <c r="H77" s="76" t="s">
+        <v>178</v>
+      </c>
+      <c r="J77" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="K77" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="L77" s="50" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="78" ht="14.25">
-      <c r="A78" s="35"/>
-      <c r="B78" s="50"/>
-      <c r="C78" s="35"/>
-      <c r="D78" s="35"/>
-      <c r="E78" s="35"/>
-      <c r="F78" s="40" t="s">
-        <v>178</v>
-      </c>
-      <c r="G78" s="40" t="s">
+      <c r="A78" s="32"/>
+      <c r="B78" s="7"/>
+      <c r="C78" s="32"/>
+      <c r="D78" s="32"/>
+      <c r="E78" s="32"/>
+      <c r="F78" s="37" t="s">
         <v>179</v>
       </c>
-      <c r="H78" s="40" t="s">
+      <c r="G78" s="37" t="s">
         <v>180</v>
       </c>
-      <c r="J78" s="40" t="s">
-        <v>178</v>
-      </c>
-      <c r="K78" s="40" t="s">
+      <c r="H78" s="37" t="s">
+        <v>181</v>
+      </c>
+      <c r="J78" s="37" t="s">
         <v>179</v>
       </c>
-      <c r="L78" s="40" t="s">
+      <c r="K78" s="37" t="s">
         <v>180</v>
       </c>
+      <c r="L78" s="37" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="79" ht="42.75" customHeight="1">
-      <c r="A79" s="63">
+      <c r="A79" s="57">
         <v>9</v>
       </c>
-      <c r="B79" s="64" t="s">
-        <v>181</v>
-      </c>
-      <c r="C79" s="65" t="s">
+      <c r="B79" s="58" t="s">
         <v>182</v>
       </c>
-      <c r="D79" s="63" t="s">
+      <c r="C79" s="57" t="s">
+        <v>183</v>
+      </c>
+      <c r="D79" s="57" t="s">
         <v>91</v>
       </c>
-      <c r="E79" s="66" t="s">
+      <c r="E79" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="F79" s="71" t="s">
-        <v>183</v>
-      </c>
-      <c r="G79" s="71" t="s">
+      <c r="F79" s="62" t="s">
         <v>184</v>
       </c>
-      <c r="H79" s="71" t="s">
+      <c r="G79" s="62" t="s">
         <v>185</v>
       </c>
-      <c r="J79" s="94" t="s">
+      <c r="H79" s="62" t="s">
         <v>186</v>
       </c>
-      <c r="K79" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="L79" s="94" t="s">
+      <c r="J79" s="80" t="s">
         <v>187</v>
       </c>
+      <c r="K79" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="L79" s="80" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="80" ht="14.25">
-      <c r="A80" s="35"/>
-      <c r="B80" s="50"/>
-      <c r="C80" s="35"/>
-      <c r="D80" s="35"/>
-      <c r="E80" s="35"/>
-      <c r="F80" s="40" t="s">
-        <v>188</v>
-      </c>
-      <c r="G80" s="40" t="s">
+      <c r="A80" s="32"/>
+      <c r="B80" s="7"/>
+      <c r="C80" s="32"/>
+      <c r="D80" s="32"/>
+      <c r="E80" s="32"/>
+      <c r="F80" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="H80" s="40" t="s">
+      <c r="G80" s="37" t="s">
         <v>190</v>
       </c>
-      <c r="J80" s="40" t="s">
-        <v>188</v>
-      </c>
-      <c r="K80" s="40" t="s">
+      <c r="H80" s="37" t="s">
+        <v>191</v>
+      </c>
+      <c r="J80" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="L80" s="40" t="s">
+      <c r="K80" s="37" t="s">
         <v>190</v>
+      </c>
+      <c r="L80" s="37" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="81" ht="14.25" customHeight="1"/>
     <row r="82" ht="14.25" customHeight="1">
-      <c r="A82" s="92" t="s">
-        <v>191</v>
-      </c>
-      <c r="B82" s="93"/>
-      <c r="C82" s="13"/>
-      <c r="D82" s="13"/>
-      <c r="E82" s="13"/>
-      <c r="F82" s="13"/>
-      <c r="G82" s="13"/>
-      <c r="H82" s="14"/>
-      <c r="J82" s="12" t="s">
-        <v>191</v>
-      </c>
-      <c r="K82" s="13"/>
-      <c r="L82" s="14"/>
+      <c r="A82" s="78" t="s">
+        <v>192</v>
+      </c>
+      <c r="B82" s="79"/>
+      <c r="C82" s="11"/>
+      <c r="D82" s="11"/>
+      <c r="E82" s="11"/>
+      <c r="F82" s="11"/>
+      <c r="G82" s="11"/>
+      <c r="H82" s="12"/>
+      <c r="J82" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="K82" s="11"/>
+      <c r="L82" s="12"/>
     </row>
     <row r="83" ht="14.25" customHeight="1">
       <c r="D83"/>
     </row>
     <row r="84" ht="57" customHeight="1">
-      <c r="A84" s="95" t="s">
-        <v>192</v>
-      </c>
-      <c r="B84" s="96" t="s">
+      <c r="A84" s="81" t="s">
         <v>193</v>
       </c>
-      <c r="C84" s="20" t="s">
+      <c r="B84" s="17" t="s">
         <v>194</v>
       </c>
-      <c r="D84" s="21" t="s">
+      <c r="C84" s="18" t="s">
+        <v>195</v>
+      </c>
+      <c r="D84" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="E84" s="54" t="s">
-        <v>195</v>
-      </c>
-      <c r="F84" s="90" t="s">
+      <c r="E84" s="22" t="s">
         <v>196</v>
       </c>
-      <c r="G84" s="90" t="s">
+      <c r="F84" s="76" t="s">
         <v>197</v>
       </c>
-      <c r="H84" s="90" t="s">
+      <c r="G84" s="76" t="s">
         <v>198</v>
       </c>
-      <c r="J84" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="K84" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="L84" s="56" t="s">
+      <c r="H84" s="76" t="s">
         <v>199</v>
       </c>
+      <c r="J84" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="K84" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="L84" s="49" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="85" ht="14.25">
-      <c r="A85" s="35"/>
-      <c r="B85" s="97"/>
-      <c r="C85" s="35"/>
-      <c r="D85" s="35"/>
-      <c r="E85" s="35"/>
-      <c r="F85" s="40" t="s">
-        <v>200</v>
-      </c>
-      <c r="G85" s="40" t="s">
+      <c r="A85" s="32"/>
+      <c r="B85" s="82"/>
+      <c r="C85" s="32"/>
+      <c r="D85" s="32"/>
+      <c r="E85" s="32"/>
+      <c r="F85" s="37" t="s">
         <v>201</v>
       </c>
-      <c r="H85" s="40" t="s">
+      <c r="G85" s="37" t="s">
         <v>202</v>
       </c>
-      <c r="J85" s="40" t="s">
-        <v>200</v>
-      </c>
-      <c r="K85" s="40" t="s">
+      <c r="H85" s="37" t="s">
+        <v>203</v>
+      </c>
+      <c r="J85" s="37" t="s">
         <v>201</v>
       </c>
-      <c r="L85" s="40" t="s">
+      <c r="K85" s="37" t="s">
         <v>202</v>
       </c>
+      <c r="L85" s="37" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="86" ht="28.5" customHeight="1">
-      <c r="A86" s="63">
+      <c r="A86" s="57">
         <v>11</v>
       </c>
-      <c r="B86" s="64" t="s">
-        <v>203</v>
-      </c>
-      <c r="C86" s="65" t="s">
+      <c r="B86" s="58" t="s">
         <v>204</v>
       </c>
-      <c r="D86" s="63" t="s">
+      <c r="C86" s="57" t="s">
+        <v>205</v>
+      </c>
+      <c r="D86" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="E86" s="66" t="s">
-        <v>205</v>
-      </c>
-      <c r="F86" s="71" t="s">
+      <c r="E86" s="59" t="s">
         <v>206</v>
       </c>
-      <c r="G86" s="71" t="s">
+      <c r="F86" s="62" t="s">
+        <v>207</v>
+      </c>
+      <c r="G86" s="62" t="s">
         <v>37</v>
       </c>
-      <c r="H86" s="71" t="s">
-        <v>207</v>
-      </c>
-      <c r="J86" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="K86" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="L86" s="62" t="s">
+      <c r="H86" s="62" t="s">
+        <v>208</v>
+      </c>
+      <c r="J86" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="K86" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="L86" s="55" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="87" ht="14.25">
-      <c r="A87" s="35"/>
-      <c r="B87" s="50"/>
-      <c r="C87" s="35"/>
-      <c r="D87" s="35"/>
-      <c r="E87" s="35"/>
-      <c r="F87" s="40" t="s">
-        <v>208</v>
-      </c>
-      <c r="G87" s="40" t="s">
+      <c r="A87" s="32"/>
+      <c r="B87" s="7"/>
+      <c r="C87" s="32"/>
+      <c r="D87" s="32"/>
+      <c r="E87" s="32"/>
+      <c r="F87" s="37" t="s">
         <v>209</v>
       </c>
-      <c r="H87" s="40" t="s">
+      <c r="G87" s="37" t="s">
         <v>210</v>
       </c>
-      <c r="J87" s="40" t="s">
-        <v>208</v>
-      </c>
-      <c r="K87" s="40" t="s">
+      <c r="H87" s="37" t="s">
+        <v>211</v>
+      </c>
+      <c r="J87" s="37" t="s">
         <v>209</v>
       </c>
-      <c r="L87" s="40" t="s">
+      <c r="K87" s="37" t="s">
         <v>210</v>
       </c>
+      <c r="L87" s="37" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="88" ht="42.75" customHeight="1">
-      <c r="A88" s="21">
+      <c r="A88" s="18">
         <v>12</v>
       </c>
-      <c r="B88" s="70" t="s">
-        <v>211</v>
-      </c>
-      <c r="C88" s="20" t="s">
+      <c r="B88" s="47" t="s">
         <v>212</v>
       </c>
-      <c r="D88" s="21" t="s">
+      <c r="C88" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="D88" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="E88" s="54" t="s">
-        <v>213</v>
-      </c>
-      <c r="F88" s="90" t="s">
+      <c r="E88" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="G88" s="55" t="s">
+      <c r="F88" s="76" t="s">
+        <v>215</v>
+      </c>
+      <c r="G88" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="H88" s="90" t="s">
-        <v>215</v>
-      </c>
-      <c r="J88" s="88" t="s">
+      <c r="H88" s="76" t="s">
         <v>216</v>
       </c>
-      <c r="K88" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="L88" s="57" t="s">
+      <c r="J88" s="74" t="s">
+        <v>217</v>
+      </c>
+      <c r="K88" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="L88" s="50" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="89" ht="14.25">
-      <c r="A89" s="35"/>
-      <c r="B89" s="50"/>
-      <c r="C89" s="35"/>
-      <c r="D89" s="35"/>
-      <c r="E89" s="35"/>
-      <c r="F89" s="40" t="s">
-        <v>217</v>
-      </c>
-      <c r="G89" s="40" t="s">
-        <v>209</v>
-      </c>
-      <c r="H89" s="40" t="s">
+      <c r="A89" s="32"/>
+      <c r="B89" s="7"/>
+      <c r="C89" s="32"/>
+      <c r="D89" s="32"/>
+      <c r="E89" s="32"/>
+      <c r="F89" s="37" t="s">
         <v>218</v>
       </c>
-      <c r="J89" s="40" t="s">
-        <v>217</v>
-      </c>
-      <c r="K89" s="40" t="s">
-        <v>209</v>
-      </c>
-      <c r="L89" s="40" t="s">
+      <c r="G89" s="37" t="s">
+        <v>210</v>
+      </c>
+      <c r="H89" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="J89" s="37" t="s">
         <v>218</v>
       </c>
+      <c r="K89" s="37" t="s">
+        <v>210</v>
+      </c>
+      <c r="L89" s="37" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="90" ht="57" customHeight="1">
-      <c r="A90" s="63">
+      <c r="A90" s="57">
         <v>13</v>
       </c>
-      <c r="B90" s="64" t="s">
-        <v>219</v>
-      </c>
-      <c r="C90" s="65" t="s">
+      <c r="B90" s="58" t="s">
         <v>220</v>
       </c>
-      <c r="D90" s="63" t="s">
+      <c r="C90" s="57" t="s">
+        <v>221</v>
+      </c>
+      <c r="D90" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="E90" s="66" t="s">
-        <v>221</v>
-      </c>
-      <c r="F90" s="71" t="s">
+      <c r="E90" s="59" t="s">
         <v>222</v>
       </c>
-      <c r="G90" s="71" t="s">
+      <c r="F90" s="62" t="s">
+        <v>223</v>
+      </c>
+      <c r="G90" s="62" t="s">
         <v>37</v>
       </c>
-      <c r="H90" s="71" t="s">
-        <v>223</v>
-      </c>
-      <c r="J90" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="K90" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="L90" s="89" t="s">
+      <c r="H90" s="62" t="s">
         <v>224</v>
       </c>
+      <c r="J90" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="K90" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="L90" s="75" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="91" ht="14.25">
-      <c r="A91" s="35"/>
-      <c r="B91" s="50"/>
-      <c r="C91" s="35"/>
-      <c r="D91" s="35"/>
-      <c r="E91" s="35"/>
-      <c r="F91" s="40" t="s">
-        <v>225</v>
-      </c>
-      <c r="G91" s="40" t="s">
-        <v>209</v>
-      </c>
-      <c r="H91" s="40" t="s">
+      <c r="A91" s="32"/>
+      <c r="B91" s="7"/>
+      <c r="C91" s="32"/>
+      <c r="D91" s="32"/>
+      <c r="E91" s="32"/>
+      <c r="F91" s="37" t="s">
         <v>226</v>
       </c>
-      <c r="J91" s="40" t="s">
-        <v>225</v>
-      </c>
-      <c r="K91" s="40" t="s">
-        <v>209</v>
-      </c>
-      <c r="L91" s="40" t="s">
+      <c r="G91" s="37" t="s">
+        <v>210</v>
+      </c>
+      <c r="H91" s="37" t="s">
+        <v>227</v>
+      </c>
+      <c r="J91" s="37" t="s">
         <v>226</v>
       </c>
+      <c r="K91" s="37" t="s">
+        <v>210</v>
+      </c>
+      <c r="L91" s="37" t="s">
+        <v>227</v>
+      </c>
     </row>
     <row r="92" ht="57" customHeight="1">
-      <c r="A92" s="21">
+      <c r="A92" s="18">
         <v>14</v>
       </c>
-      <c r="B92" s="70" t="s">
-        <v>227</v>
-      </c>
-      <c r="C92" s="20" t="s">
+      <c r="B92" s="47" t="s">
         <v>228</v>
       </c>
-      <c r="D92" s="21" t="s">
+      <c r="C92" s="18" t="s">
+        <v>229</v>
+      </c>
+      <c r="D92" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="E92" s="54" t="s">
-        <v>229</v>
-      </c>
-      <c r="F92" s="90" t="s">
+      <c r="E92" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="G92" s="90" t="s">
+      <c r="F92" s="76" t="s">
         <v>231</v>
       </c>
-      <c r="H92" s="90" t="s">
+      <c r="G92" s="76" t="s">
         <v>232</v>
       </c>
-      <c r="J92" s="57" t="s">
+      <c r="H92" s="76" t="s">
         <v>233</v>
       </c>
-      <c r="K92" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="L92" s="57" t="s">
+      <c r="J92" s="50" t="s">
+        <v>234</v>
+      </c>
+      <c r="K92" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="L92" s="50" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="93" ht="14.25">
-      <c r="A93" s="35"/>
-      <c r="B93" s="50"/>
-      <c r="C93" s="35"/>
-      <c r="D93" s="35"/>
-      <c r="E93" s="35"/>
-      <c r="F93" s="40" t="s">
-        <v>234</v>
-      </c>
-      <c r="G93" s="40" t="s">
+      <c r="A93" s="32"/>
+      <c r="B93" s="7"/>
+      <c r="C93" s="32"/>
+      <c r="D93" s="32"/>
+      <c r="E93" s="32"/>
+      <c r="F93" s="37" t="s">
         <v>235</v>
       </c>
-      <c r="H93" s="40" t="s">
+      <c r="G93" s="37" t="s">
         <v>236</v>
       </c>
-      <c r="J93" s="40" t="s">
-        <v>234</v>
-      </c>
-      <c r="K93" s="40" t="s">
+      <c r="H93" s="37" t="s">
+        <v>237</v>
+      </c>
+      <c r="J93" s="37" t="s">
         <v>235</v>
       </c>
-      <c r="L93" s="40" t="s">
+      <c r="K93" s="37" t="s">
         <v>236</v>
       </c>
+      <c r="L93" s="37" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="94" ht="42.75" customHeight="1">
-      <c r="A94" s="63">
+      <c r="A94" s="57">
         <v>15</v>
       </c>
-      <c r="B94" s="64" t="s">
-        <v>237</v>
-      </c>
-      <c r="C94" s="65" t="s">
+      <c r="B94" s="58" t="s">
         <v>238</v>
       </c>
-      <c r="D94" s="63" t="s">
+      <c r="C94" s="57" t="s">
+        <v>239</v>
+      </c>
+      <c r="D94" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="E94" s="66" t="s">
+      <c r="E94" s="59" t="s">
         <v>123</v>
       </c>
-      <c r="F94" s="71" t="s">
-        <v>239</v>
-      </c>
-      <c r="G94" s="71" t="s">
+      <c r="F94" s="62" t="s">
         <v>240</v>
       </c>
-      <c r="H94" s="71" t="s">
-        <v>240</v>
-      </c>
-      <c r="J94" s="89" t="s">
+      <c r="G94" s="62" t="s">
         <v>241</v>
       </c>
-      <c r="K94" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="L94" s="89" t="s">
+      <c r="H94" s="62" t="s">
+        <v>241</v>
+      </c>
+      <c r="J94" s="75" t="s">
         <v>242</v>
       </c>
+      <c r="K94" s="55" t="s">
+        <v>20</v>
+      </c>
+      <c r="L94" s="75" t="s">
+        <v>243</v>
+      </c>
     </row>
     <row r="95" ht="14.25">
-      <c r="A95" s="35"/>
-      <c r="B95" s="50"/>
-      <c r="C95" s="35"/>
-      <c r="D95" s="35"/>
-      <c r="E95" s="35"/>
-      <c r="F95" s="40" t="s">
-        <v>243</v>
-      </c>
-      <c r="G95" s="40" t="s">
+      <c r="A95" s="32"/>
+      <c r="B95" s="7"/>
+      <c r="C95" s="32"/>
+      <c r="D95" s="32"/>
+      <c r="E95" s="32"/>
+      <c r="F95" s="37" t="s">
         <v>244</v>
       </c>
-      <c r="H95" s="40" t="s">
+      <c r="G95" s="37" t="s">
         <v>245</v>
       </c>
-      <c r="J95" s="40" t="s">
-        <v>243</v>
-      </c>
-      <c r="K95" s="40" t="s">
+      <c r="H95" s="37" t="s">
+        <v>246</v>
+      </c>
+      <c r="J95" s="37" t="s">
         <v>244</v>
       </c>
-      <c r="L95" s="40" t="s">
+      <c r="K95" s="37" t="s">
         <v>245</v>
+      </c>
+      <c r="L95" s="37" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="96" ht="14.25">
       <c r="A96" s="1"/>
-      <c r="B96" s="82"/>
+      <c r="B96" s="1"/>
     </row>
     <row r="97" ht="14.25" customHeight="1">
-      <c r="A97" s="98" t="s">
-        <v>246</v>
-      </c>
-      <c r="B97" s="99"/>
-      <c r="C97" s="100"/>
-      <c r="D97" s="100"/>
-      <c r="E97" s="100"/>
-      <c r="F97" s="100"/>
-      <c r="G97" s="100"/>
-      <c r="H97" s="101"/>
-      <c r="J97" s="12" t="s">
-        <v>246</v>
-      </c>
-      <c r="K97" s="13"/>
-      <c r="L97" s="14"/>
+      <c r="A97" s="83" t="s">
+        <v>247</v>
+      </c>
+      <c r="B97" s="84"/>
+      <c r="C97" s="85"/>
+      <c r="D97" s="85"/>
+      <c r="E97" s="85"/>
+      <c r="F97" s="85"/>
+      <c r="G97" s="85"/>
+      <c r="H97" s="86"/>
+      <c r="J97" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="K97" s="11"/>
+      <c r="L97" s="12"/>
     </row>
     <row r="98" ht="14.25" customHeight="1">
-      <c r="A98" s="102"/>
-      <c r="B98" s="82"/>
+      <c r="A98" s="87"/>
+      <c r="B98" s="1"/>
       <c r="D98"/>
     </row>
     <row r="99" ht="57" customHeight="1">
-      <c r="A99" s="103" t="s">
-        <v>192</v>
-      </c>
-      <c r="B99" s="104" t="s">
-        <v>247</v>
-      </c>
-      <c r="C99" s="105" t="s">
-        <v>194</v>
-      </c>
-      <c r="D99" s="106" t="s">
+      <c r="A99" s="88" t="s">
+        <v>193</v>
+      </c>
+      <c r="B99" s="89" t="s">
+        <v>248</v>
+      </c>
+      <c r="C99" s="88" t="s">
+        <v>195</v>
+      </c>
+      <c r="D99" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="E99" s="107" t="s">
-        <v>195</v>
-      </c>
-      <c r="F99" s="90" t="s">
-        <v>248</v>
-      </c>
-      <c r="G99" s="90" t="s">
+      <c r="E99" s="91" t="s">
+        <v>196</v>
+      </c>
+      <c r="F99" s="76" t="s">
         <v>249</v>
       </c>
-      <c r="H99" s="90" t="s">
+      <c r="G99" s="76" t="s">
         <v>250</v>
       </c>
-      <c r="J99" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="K99" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="L99" s="25" t="s">
+      <c r="H99" s="76" t="s">
+        <v>251</v>
+      </c>
+      <c r="J99" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K99" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="L99" s="22" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="100" ht="14.25">
-      <c r="A100" s="35"/>
-      <c r="B100" s="97"/>
-      <c r="C100" s="35"/>
-      <c r="D100" s="35"/>
-      <c r="E100" s="35"/>
-      <c r="F100" s="40" t="s">
-        <v>251</v>
-      </c>
-      <c r="G100" s="40" t="s">
+      <c r="A100" s="32"/>
+      <c r="B100" s="82"/>
+      <c r="C100" s="32"/>
+      <c r="D100" s="32"/>
+      <c r="E100" s="32"/>
+      <c r="F100" s="37" t="s">
         <v>252</v>
       </c>
-      <c r="H100" s="40" t="s">
+      <c r="G100" s="37" t="s">
         <v>253</v>
       </c>
-      <c r="J100" s="40" t="s">
-        <v>251</v>
-      </c>
-      <c r="K100" s="40" t="s">
+      <c r="H100" s="37" t="s">
+        <v>254</v>
+      </c>
+      <c r="J100" s="37" t="s">
         <v>252</v>
       </c>
-      <c r="L100" s="40" t="s">
+      <c r="K100" s="37" t="s">
         <v>253</v>
       </c>
+      <c r="L100" s="37" t="s">
+        <v>254</v>
+      </c>
     </row>
     <row r="101" ht="57" customHeight="1">
-      <c r="A101" s="108" t="s">
-        <v>254</v>
-      </c>
-      <c r="B101" s="109" t="s">
+      <c r="A101" s="92" t="s">
         <v>255</v>
       </c>
-      <c r="C101" s="110" t="s">
-        <v>238</v>
-      </c>
-      <c r="D101" s="63" t="s">
+      <c r="B101" s="93" t="s">
+        <v>256</v>
+      </c>
+      <c r="C101" s="94" t="s">
+        <v>239</v>
+      </c>
+      <c r="D101" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="E101" s="66" t="s">
+      <c r="E101" s="59" t="s">
         <v>123</v>
       </c>
-      <c r="F101" s="71" t="s">
-        <v>256</v>
-      </c>
-      <c r="G101" s="71" t="s">
+      <c r="F101" s="62" t="s">
         <v>257</v>
       </c>
-      <c r="H101" s="71" t="s">
-        <v>257</v>
-      </c>
-      <c r="J101" s="111" t="s">
-        <v>241</v>
-      </c>
-      <c r="K101" s="49" t="s">
-        <v>20</v>
-      </c>
-      <c r="L101" s="111" t="s">
+      <c r="G101" s="62" t="s">
+        <v>258</v>
+      </c>
+      <c r="H101" s="62" t="s">
+        <v>258</v>
+      </c>
+      <c r="J101" s="95" t="s">
         <v>242</v>
       </c>
+      <c r="K101" s="44" t="s">
+        <v>20</v>
+      </c>
+      <c r="L101" s="95" t="s">
+        <v>243</v>
+      </c>
     </row>
     <row r="102" ht="14.25" customHeight="1">
-      <c r="A102" s="81"/>
-      <c r="B102" s="97"/>
-      <c r="C102" s="35"/>
-      <c r="D102" s="35"/>
-      <c r="E102" s="35"/>
-      <c r="F102" s="40" t="s">
-        <v>258</v>
-      </c>
-      <c r="G102" s="40" t="s">
+      <c r="A102" s="67"/>
+      <c r="B102" s="82"/>
+      <c r="C102" s="32"/>
+      <c r="D102" s="32"/>
+      <c r="E102" s="32"/>
+      <c r="F102" s="37" t="s">
         <v>259</v>
       </c>
-      <c r="H102" s="40" t="s">
+      <c r="G102" s="37" t="s">
         <v>260</v>
       </c>
-      <c r="J102" s="40" t="s">
-        <v>258</v>
-      </c>
-      <c r="K102" s="40" t="s">
+      <c r="H102" s="37" t="s">
+        <v>261</v>
+      </c>
+      <c r="J102" s="37" t="s">
         <v>259</v>
       </c>
-      <c r="L102" s="40" t="s">
+      <c r="K102" s="37" t="s">
         <v>260</v>
       </c>
+      <c r="L102" s="37" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="104" ht="14.25" customHeight="1">
-      <c r="A104" s="92" t="s">
-        <v>261</v>
-      </c>
-      <c r="B104" s="93"/>
-      <c r="C104" s="13"/>
-      <c r="D104" s="13"/>
-      <c r="E104" s="13"/>
-      <c r="F104" s="13"/>
-      <c r="G104" s="13"/>
-      <c r="H104" s="14"/>
-      <c r="J104" s="12" t="s">
-        <v>261</v>
-      </c>
-      <c r="K104" s="13"/>
-      <c r="L104" s="14"/>
+      <c r="A104" s="78" t="s">
+        <v>262</v>
+      </c>
+      <c r="B104" s="79"/>
+      <c r="C104" s="11"/>
+      <c r="D104" s="11"/>
+      <c r="E104" s="11"/>
+      <c r="F104" s="11"/>
+      <c r="G104" s="11"/>
+      <c r="H104" s="12"/>
+      <c r="J104" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="K104" s="11"/>
+      <c r="L104" s="12"/>
     </row>
     <row r="106" ht="74.25" customHeight="1">
-      <c r="A106" s="21">
+      <c r="A106" s="18">
         <v>16</v>
       </c>
-      <c r="B106" s="70" t="s">
-        <v>262</v>
-      </c>
-      <c r="C106" s="20" t="s">
+      <c r="B106" s="47" t="s">
         <v>263</v>
       </c>
-      <c r="D106" s="21" t="s">
+      <c r="C106" s="18" t="s">
+        <v>264</v>
+      </c>
+      <c r="D106" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="E106" s="25" t="s">
-        <v>264</v>
-      </c>
-      <c r="F106" s="90" t="s">
+      <c r="E106" s="22" t="s">
         <v>265</v>
       </c>
-      <c r="G106" s="90" t="s">
+      <c r="F106" s="76" t="s">
         <v>266</v>
       </c>
-      <c r="H106" s="90" t="s">
-        <v>266</v>
-      </c>
-      <c r="J106" s="25" t="s">
-        <v>20</v>
-      </c>
-      <c r="K106" s="90" t="s">
+      <c r="G106" s="76" t="s">
         <v>267</v>
       </c>
-      <c r="L106" s="90" t="s">
+      <c r="H106" s="76" t="s">
+        <v>267</v>
+      </c>
+      <c r="J106" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K106" s="76" t="s">
         <v>268</v>
       </c>
+      <c r="L106" s="76" t="s">
+        <v>269</v>
+      </c>
     </row>
     <row r="107" ht="14.25" customHeight="1">
-      <c r="A107" s="35"/>
-      <c r="B107" s="50"/>
-      <c r="C107" s="35"/>
-      <c r="D107" s="35"/>
-      <c r="E107" s="35"/>
-      <c r="F107" s="40" t="s">
-        <v>269</v>
-      </c>
-      <c r="G107" s="40" t="s">
+      <c r="A107" s="32"/>
+      <c r="B107" s="7"/>
+      <c r="C107" s="32"/>
+      <c r="D107" s="32"/>
+      <c r="E107" s="32"/>
+      <c r="F107" s="37" t="s">
         <v>270</v>
       </c>
-      <c r="H107" s="40" t="s">
+      <c r="G107" s="37" t="s">
         <v>271</v>
       </c>
-      <c r="J107" s="40" t="s">
-        <v>269</v>
-      </c>
-      <c r="K107" s="40" t="s">
+      <c r="H107" s="37" t="s">
+        <v>272</v>
+      </c>
+      <c r="J107" s="37" t="s">
         <v>270</v>
       </c>
-      <c r="L107" s="40" t="s">
+      <c r="K107" s="37" t="s">
         <v>271</v>
+      </c>
+      <c r="L107" s="37" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="108" ht="14.25" customHeight="1">
       <c r="A108" t="s">
-        <v>272</v>
-      </c>
-      <c r="B108" s="112"/>
+        <v>273</v>
+      </c>
+      <c r="B108" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="245">

</xml_diff>